<commit_message>
Ajout du cout annuel projete pour la saison 2027-2028
Reprise du fichier annote par Thibault Duchene : taux cibles 2026-27
remplis et nouvelle colonne des taux apres formation pour 2027-28.

Ajouts :
- colonne "Cout annuel 2027-28" = heures x taux 2027-28 x 28 semaines
- total club et ligne "Ecart vs cible 2026-27"
- note sur l'hypothese de volume d'heures constant entre les deux saisons

Resultats : 146 398 EUR aujourd'hui, 150 304 EUR avec les cibles
2026-27, 159 264 EUR en 2027-28 apres formation.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CP9eZ8ypAHjVkDVd1FLqef
</commit_message>
<xml_diff>
--- a/Horaires profs 2026-2027/Couts professeurs 2026-2027.xlsx
+++ b/Horaires profs 2026-2027/Couts professeurs 2026-2027.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Coûts profs'!$9:$9</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Coûts profs'!$A$9:$I$31</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Coûts profs'!$A$9:$K$31</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,9 +24,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
-  <si>
-    <t xml:space="preserve">Coût des professeurs — Cycle annuel 2026-2027</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+  <si>
+    <t xml:space="preserve">Coût des professeurs — cycle 2026-2027 et projection 2027-2028</t>
   </si>
   <si>
     <t xml:space="preserve">Cours collectifs uniquement. Les cellules bleues et jaunes se modifient, les noires sont calculées.</t>
@@ -72,11 +72,19 @@
   </si>
   <si>
     <t xml:space="preserve">Taux ciblé
-(€/h)</t>
+2026-27 (€/h)</t>
   </si>
   <si>
     <t xml:space="preserve">Coût annuel
-ciblé</t>
+ciblé 2026-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux après format.
+2027-28 (€/h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coût annuel
+2027-28</t>
   </si>
   <si>
     <t xml:space="preserve">Taha Yassine</t>
@@ -151,6 +159,9 @@
     <t xml:space="preserve">Écart vs actuel</t>
   </si>
   <si>
+    <t xml:space="preserve">Écart vs ciblé 2026-27</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
@@ -163,10 +174,13 @@
     <t xml:space="preserve">• Un prof encadrant plusieurs groupes en même temps ne voit cette heure comptée qu'une fois.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Coûts horaires : saisis par Thibault Duchêne, non issus d'iClub.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Colonne « Taux ciblé » : laissez vide pour garder le taux actuel, ou indiquez le nouveau taux horaire — le coût annuel ciblé se met à jour.</t>
+    <t xml:space="preserve">• Coûts horaires actuels, taux ciblés 2026-27 et taux après formation 2027-28 : saisis par Thibault Duchêne, non issus d'iClub.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Coût annuel 2027-28 : calculé sur le MÊME volume d'heures qu'en 2026-27 et les mêmes 28 semaines. Si les horaires changent pour 2027-28, il faudra réextraire iClub et mettre la colonne B à jour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Taux ciblé et taux 2027-28 : si la case est laissée vide, le calcul reprend le taux de la colonne précédente (ciblé, sinon actuel).</t>
   </si>
   <si>
     <t xml:space="preserve">• Scénario A (+2 €/h) est une hausse uniforme en valeur ; scénario B (+10 %) est proportionnelle. Les deux ne frappent donc pas les mêmes profs de la même façon.</t>
@@ -178,7 +192,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0&quot; semaines&quot;"/>
+    <numFmt numFmtId="165" formatCode="0&quot; sem.&quot;"/>
     <numFmt numFmtId="166" formatCode="\+0&quot; €/h&quot;"/>
     <numFmt numFmtId="167" formatCode="\+0\ %"/>
     <numFmt numFmtId="168" formatCode="0.0&quot; h&quot;"/>
@@ -293,7 +307,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -310,6 +324,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E5C94"/>
+        <bgColor rgb="FF595959"/>
       </patternFill>
     </fill>
     <fill>
@@ -395,7 +415,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -436,27 +456,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -468,14 +492,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="170" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -516,7 +532,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -529,7 +545,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -573,6 +589,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2E5C94"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -634,7 +658,7 @@
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF2E5C94"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
@@ -825,16 +849,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -876,7 +900,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
         <v>6</v>
       </c>
@@ -904,803 +928,1040 @@
       <c r="I9" s="9" t="s">
         <v>14</v>
       </c>
+      <c r="J9" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="11" t="n">
+      <c r="A10" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="12" t="n">
         <v>31.5</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <f aca="false">B10*C10</f>
         <v>945</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="15" t="n">
         <f aca="false">D10*$B$5</f>
         <v>26460</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="16" t="n">
         <f aca="false">B10*(C10+$B$6)*$B$5</f>
         <v>28224</v>
       </c>
-      <c r="G10" s="15" t="n">
+      <c r="G10" s="16" t="n">
         <f aca="false">E10*(1+$B$7)</f>
         <v>29106</v>
       </c>
-      <c r="H10" s="16"/>
+      <c r="H10" s="17" t="n">
+        <v>30</v>
+      </c>
       <c r="I10" s="15" t="n">
         <f aca="false">B10*IF(H10="",C10,H10)*$B$5</f>
         <v>26460</v>
       </c>
+      <c r="J10" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="K10" s="15" t="n">
+        <f aca="false">B10*IF(J10="",IF(H10="",C10,H10),J10)*$B$5</f>
+        <v>30870</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="C11" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D11" s="20" t="n">
+      <c r="A11" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D11" s="19" t="n">
         <f aca="false">B11*C11</f>
         <v>729</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="20" t="n">
         <f aca="false">D11*$B$5</f>
         <v>20412</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F11" s="21" t="n">
         <f aca="false">B11*(C11+$B$6)*$B$5</f>
         <v>21924</v>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="G11" s="21" t="n">
         <f aca="false">E11*(1+$B$7)</f>
         <v>22453.2</v>
       </c>
-      <c r="H11" s="16"/>
-      <c r="I11" s="22" t="n">
+      <c r="H11" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="I11" s="20" t="n">
         <f aca="false">B11*IF(H11="",C11,H11)*$B$5</f>
         <v>20412</v>
       </c>
+      <c r="J11" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K11" s="20" t="n">
+        <f aca="false">B11*IF(J11="",IF(H11="",C11,H11),J11)*$B$5</f>
+        <v>22680</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="11" t="n">
+      <c r="A12" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="C12" s="12" t="n">
-        <v>27</v>
-      </c>
-      <c r="D12" s="13" t="n">
+      <c r="C12" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D12" s="14" t="n">
         <f aca="false">B12*C12</f>
         <v>702</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <f aca="false">D12*$B$5</f>
         <v>19656</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="16" t="n">
         <f aca="false">B12*(C12+$B$6)*$B$5</f>
         <v>21112</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="16" t="n">
         <f aca="false">E12*(1+$B$7)</f>
         <v>21621.6</v>
       </c>
-      <c r="H12" s="16"/>
+      <c r="H12" s="17" t="n">
+        <v>27</v>
+      </c>
       <c r="I12" s="15" t="n">
         <f aca="false">B12*IF(H12="",C12,H12)*$B$5</f>
         <v>19656</v>
       </c>
+      <c r="J12" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K12" s="15" t="n">
+        <f aca="false">B12*IF(J12="",IF(H12="",C12,H12),J12)*$B$5</f>
+        <v>19656</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="18" t="n">
+      <c r="A13" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C13" s="13" t="n">
         <v>35</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="19" t="n">
         <f aca="false">B13*C13</f>
         <v>875</v>
       </c>
-      <c r="E13" s="21" t="n">
+      <c r="E13" s="20" t="n">
         <f aca="false">D13*$B$5</f>
         <v>24500</v>
       </c>
-      <c r="F13" s="22" t="n">
+      <c r="F13" s="21" t="n">
         <f aca="false">B13*(C13+$B$6)*$B$5</f>
         <v>25900</v>
       </c>
-      <c r="G13" s="22" t="n">
+      <c r="G13" s="21" t="n">
         <f aca="false">E13*(1+$B$7)</f>
         <v>26950</v>
       </c>
-      <c r="H13" s="16"/>
-      <c r="I13" s="22" t="n">
+      <c r="H13" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="I13" s="20" t="n">
         <f aca="false">B13*IF(H13="",C13,H13)*$B$5</f>
-        <v>24500</v>
+        <v>25900</v>
+      </c>
+      <c r="J13" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="K13" s="20" t="n">
+        <f aca="false">B13*IF(J13="",IF(H13="",C13,H13),J13)*$B$5</f>
+        <v>25900</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="11" t="n">
+      <c r="A14" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">B14*C14</f>
         <v>425</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="15" t="n">
         <f aca="false">D14*$B$5</f>
         <v>11900</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="16" t="n">
         <f aca="false">B14*(C14+$B$6)*$B$5</f>
         <v>12852</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="16" t="n">
         <f aca="false">E14*(1+$B$7)</f>
         <v>13090</v>
       </c>
-      <c r="H14" s="16"/>
+      <c r="H14" s="17" t="n">
+        <v>27</v>
+      </c>
       <c r="I14" s="15" t="n">
         <f aca="false">B14*IF(H14="",C14,H14)*$B$5</f>
-        <v>11900</v>
+        <v>12852</v>
+      </c>
+      <c r="J14" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K14" s="15" t="n">
+        <f aca="false">B14*IF(J14="",IF(H14="",C14,H14),J14)*$B$5</f>
+        <v>14280</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="18" t="n">
+      <c r="A15" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="12" t="n">
         <v>6.5</v>
       </c>
-      <c r="C15" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D15" s="20" t="n">
+      <c r="C15" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D15" s="19" t="n">
         <f aca="false">B15*C15</f>
         <v>175.5</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="20" t="n">
         <f aca="false">D15*$B$5</f>
         <v>4914</v>
       </c>
-      <c r="F15" s="22" t="n">
+      <c r="F15" s="21" t="n">
         <f aca="false">B15*(C15+$B$6)*$B$5</f>
         <v>5278</v>
       </c>
-      <c r="G15" s="22" t="n">
+      <c r="G15" s="21" t="n">
         <f aca="false">E15*(1+$B$7)</f>
         <v>5405.4</v>
       </c>
-      <c r="H15" s="16"/>
-      <c r="I15" s="22" t="n">
+      <c r="H15" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" s="20" t="n">
         <f aca="false">B15*IF(H15="",C15,H15)*$B$5</f>
-        <v>4914</v>
+        <v>5460</v>
+      </c>
+      <c r="J15" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K15" s="20" t="n">
+        <f aca="false">B15*IF(J15="",IF(H15="",C15,H15),J15)*$B$5</f>
+        <v>5460</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="11" t="n">
+      <c r="A16" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="12" t="n">
         <v>5.5</v>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <f aca="false">B16*C16</f>
         <v>275</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="15" t="n">
         <f aca="false">D16*$B$5</f>
         <v>7700</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="16" t="n">
         <f aca="false">B16*(C16+$B$6)*$B$5</f>
         <v>8008</v>
       </c>
-      <c r="G16" s="15" t="n">
+      <c r="G16" s="16" t="n">
         <f aca="false">E16*(1+$B$7)</f>
         <v>8470</v>
       </c>
-      <c r="H16" s="16"/>
+      <c r="H16" s="17" t="n">
+        <v>50</v>
+      </c>
       <c r="I16" s="15" t="n">
         <f aca="false">B16*IF(H16="",C16,H16)*$B$5</f>
         <v>7700</v>
       </c>
+      <c r="J16" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="K16" s="15" t="n">
+        <f aca="false">B16*IF(J16="",IF(H16="",C16,H16),J16)*$B$5</f>
+        <v>7700</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="18" t="n">
+      <c r="A17" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="19" t="n">
         <f aca="false">B17*C17</f>
         <v>125</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="20" t="n">
         <f aca="false">D17*$B$5</f>
         <v>3500</v>
       </c>
-      <c r="F17" s="22" t="n">
+      <c r="F17" s="21" t="n">
         <f aca="false">B17*(C17+$B$6)*$B$5</f>
         <v>3780</v>
       </c>
-      <c r="G17" s="22" t="n">
+      <c r="G17" s="21" t="n">
         <f aca="false">E17*(1+$B$7)</f>
         <v>3850</v>
       </c>
-      <c r="H17" s="16"/>
-      <c r="I17" s="22" t="n">
+      <c r="H17" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="I17" s="20" t="n">
         <f aca="false">B17*IF(H17="",C17,H17)*$B$5</f>
-        <v>3500</v>
+        <v>3780</v>
+      </c>
+      <c r="J17" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K17" s="20" t="n">
+        <f aca="false">B17*IF(J17="",IF(H17="",C17,H17),J17)*$B$5</f>
+        <v>3780</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="11" t="n">
+      <c r="A18" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="12" t="n">
         <v>4.5</v>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="14" t="n">
         <f aca="false">B18*C18</f>
         <v>112.5</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E18" s="15" t="n">
         <f aca="false">D18*$B$5</f>
         <v>3150</v>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="16" t="n">
         <f aca="false">B18*(C18+$B$6)*$B$5</f>
         <v>3402</v>
       </c>
-      <c r="G18" s="15" t="n">
+      <c r="G18" s="16" t="n">
         <f aca="false">E18*(1+$B$7)</f>
         <v>3465</v>
       </c>
-      <c r="H18" s="16"/>
+      <c r="H18" s="17" t="n">
+        <v>25</v>
+      </c>
       <c r="I18" s="15" t="n">
         <f aca="false">B18*IF(H18="",C18,H18)*$B$5</f>
         <v>3150</v>
       </c>
+      <c r="J18" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K18" s="15" t="n">
+        <f aca="false">B18*IF(J18="",IF(H18="",C18,H18),J18)*$B$5</f>
+        <v>3402</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="18" t="n">
+      <c r="A19" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="12" t="n">
         <v>4.5</v>
       </c>
-      <c r="C19" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D19" s="20" t="n">
+      <c r="C19" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D19" s="19" t="n">
         <f aca="false">B19*C19</f>
         <v>121.5</v>
       </c>
-      <c r="E19" s="21" t="n">
+      <c r="E19" s="20" t="n">
         <f aca="false">D19*$B$5</f>
         <v>3402</v>
       </c>
-      <c r="F19" s="22" t="n">
+      <c r="F19" s="21" t="n">
         <f aca="false">B19*(C19+$B$6)*$B$5</f>
         <v>3654</v>
       </c>
-      <c r="G19" s="22" t="n">
+      <c r="G19" s="21" t="n">
         <f aca="false">E19*(1+$B$7)</f>
         <v>3742.2</v>
       </c>
-      <c r="H19" s="16"/>
-      <c r="I19" s="22" t="n">
+      <c r="H19" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="I19" s="20" t="n">
         <f aca="false">B19*IF(H19="",C19,H19)*$B$5</f>
         <v>3402</v>
       </c>
+      <c r="J19" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K19" s="20" t="n">
+        <f aca="false">B19*IF(J19="",IF(H19="",C19,H19),J19)*$B$5</f>
+        <v>3780</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="11" t="n">
+      <c r="A20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="12" t="n">
         <v>4.5</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="D20" s="13" t="n">
+      <c r="D20" s="14" t="n">
         <f aca="false">B20*C20</f>
         <v>135</v>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="E20" s="15" t="n">
         <f aca="false">D20*$B$5</f>
         <v>3780</v>
       </c>
-      <c r="F20" s="15" t="n">
+      <c r="F20" s="16" t="n">
         <f aca="false">B20*(C20+$B$6)*$B$5</f>
         <v>4032</v>
       </c>
-      <c r="G20" s="15" t="n">
+      <c r="G20" s="16" t="n">
         <f aca="false">E20*(1+$B$7)</f>
         <v>4158</v>
       </c>
-      <c r="H20" s="16"/>
+      <c r="H20" s="17" t="n">
+        <v>30</v>
+      </c>
       <c r="I20" s="15" t="n">
         <f aca="false">B20*IF(H20="",C20,H20)*$B$5</f>
         <v>3780</v>
       </c>
+      <c r="J20" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K20" s="15" t="n">
+        <f aca="false">B20*IF(J20="",IF(H20="",C20,H20),J20)*$B$5</f>
+        <v>3780</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="18" t="n">
+      <c r="A21" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="12" t="n">
         <v>3.5</v>
       </c>
-      <c r="C21" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D21" s="20" t="n">
+      <c r="C21" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D21" s="19" t="n">
         <f aca="false">B21*C21</f>
         <v>94.5</v>
       </c>
-      <c r="E21" s="21" t="n">
+      <c r="E21" s="20" t="n">
         <f aca="false">D21*$B$5</f>
         <v>2646</v>
       </c>
-      <c r="F21" s="22" t="n">
+      <c r="F21" s="21" t="n">
         <f aca="false">B21*(C21+$B$6)*$B$5</f>
         <v>2842</v>
       </c>
-      <c r="G21" s="22" t="n">
+      <c r="G21" s="21" t="n">
         <f aca="false">E21*(1+$B$7)</f>
         <v>2910.6</v>
       </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="22" t="n">
+      <c r="H21" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="I21" s="20" t="n">
         <f aca="false">B21*IF(H21="",C21,H21)*$B$5</f>
         <v>2646</v>
       </c>
+      <c r="J21" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K21" s="20" t="n">
+        <f aca="false">B21*IF(J21="",IF(H21="",C21,H21),J21)*$B$5</f>
+        <v>2646</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="11" t="n">
+      <c r="A22" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="13" t="n">
         <v>35</v>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="14" t="n">
         <f aca="false">B22*C22</f>
         <v>105</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="15" t="n">
         <f aca="false">D22*$B$5</f>
         <v>2940</v>
       </c>
-      <c r="F22" s="15" t="n">
+      <c r="F22" s="16" t="n">
         <f aca="false">B22*(C22+$B$6)*$B$5</f>
         <v>3108</v>
       </c>
-      <c r="G22" s="15" t="n">
+      <c r="G22" s="16" t="n">
         <f aca="false">E22*(1+$B$7)</f>
         <v>3234</v>
       </c>
-      <c r="H22" s="16"/>
+      <c r="H22" s="17" t="n">
+        <v>37</v>
+      </c>
       <c r="I22" s="15" t="n">
         <f aca="false">B22*IF(H22="",C22,H22)*$B$5</f>
-        <v>2940</v>
+        <v>3108</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="K22" s="15" t="n">
+        <f aca="false">B22*IF(J22="",IF(H22="",C22,H22),J22)*$B$5</f>
+        <v>3108</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="18" t="n">
+      <c r="A23" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D23" s="20" t="n">
+      <c r="C23" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D23" s="19" t="n">
         <f aca="false">B23*C23</f>
         <v>81</v>
       </c>
-      <c r="E23" s="21" t="n">
+      <c r="E23" s="20" t="n">
         <f aca="false">D23*$B$5</f>
         <v>2268</v>
       </c>
-      <c r="F23" s="22" t="n">
+      <c r="F23" s="21" t="n">
         <f aca="false">B23*(C23+$B$6)*$B$5</f>
         <v>2436</v>
       </c>
-      <c r="G23" s="22" t="n">
+      <c r="G23" s="21" t="n">
         <f aca="false">E23*(1+$B$7)</f>
         <v>2494.8</v>
       </c>
-      <c r="H23" s="16"/>
-      <c r="I23" s="22" t="n">
+      <c r="H23" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="I23" s="20" t="n">
         <f aca="false">B23*IF(H23="",C23,H23)*$B$5</f>
         <v>2268</v>
       </c>
+      <c r="J23" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K23" s="20" t="n">
+        <f aca="false">B23*IF(J23="",IF(H23="",C23,H23),J23)*$B$5</f>
+        <v>2268</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="11" t="n">
+      <c r="A24" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="12" t="n">
         <v>2.5</v>
       </c>
-      <c r="C24" s="12" t="n">
-        <v>27</v>
-      </c>
-      <c r="D24" s="13" t="n">
+      <c r="C24" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="D24" s="14" t="n">
         <f aca="false">B24*C24</f>
         <v>67.5</v>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="E24" s="15" t="n">
         <f aca="false">D24*$B$5</f>
         <v>1890</v>
       </c>
-      <c r="F24" s="15" t="n">
+      <c r="F24" s="16" t="n">
         <f aca="false">B24*(C24+$B$6)*$B$5</f>
         <v>2030</v>
       </c>
-      <c r="G24" s="15" t="n">
+      <c r="G24" s="16" t="n">
         <f aca="false">E24*(1+$B$7)</f>
         <v>2079</v>
       </c>
-      <c r="H24" s="16"/>
+      <c r="H24" s="17" t="n">
+        <v>27</v>
+      </c>
       <c r="I24" s="15" t="n">
         <f aca="false">B24*IF(H24="",C24,H24)*$B$5</f>
         <v>1890</v>
       </c>
+      <c r="J24" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K24" s="15" t="n">
+        <f aca="false">B24*IF(J24="",IF(H24="",C24,H24),J24)*$B$5</f>
+        <v>1890</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="18" t="n">
+      <c r="A25" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C25" s="13" t="n">
         <v>21</v>
       </c>
-      <c r="D25" s="20" t="n">
+      <c r="D25" s="19" t="n">
         <f aca="false">B25*C25</f>
         <v>42</v>
       </c>
-      <c r="E25" s="21" t="n">
+      <c r="E25" s="20" t="n">
         <f aca="false">D25*$B$5</f>
         <v>1176</v>
       </c>
-      <c r="F25" s="22" t="n">
+      <c r="F25" s="21" t="n">
         <f aca="false">B25*(C25+$B$6)*$B$5</f>
         <v>1288</v>
       </c>
-      <c r="G25" s="22" t="n">
+      <c r="G25" s="21" t="n">
         <f aca="false">E25*(1+$B$7)</f>
         <v>1293.6</v>
       </c>
-      <c r="H25" s="16"/>
-      <c r="I25" s="22" t="n">
+      <c r="H25" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="I25" s="20" t="n">
         <f aca="false">B25*IF(H25="",C25,H25)*$B$5</f>
-        <v>1176</v>
+        <v>1288</v>
+      </c>
+      <c r="J25" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="K25" s="20" t="n">
+        <f aca="false">B25*IF(J25="",IF(H25="",C25,H25),J25)*$B$5</f>
+        <v>1400</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="11" t="n">
+      <c r="A26" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C26" s="12" t="n">
+      <c r="C26" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D26" s="13" t="n">
+      <c r="D26" s="14" t="n">
         <f aca="false">B26*C26</f>
         <v>50</v>
       </c>
-      <c r="E26" s="14" t="n">
+      <c r="E26" s="15" t="n">
         <f aca="false">D26*$B$5</f>
         <v>1400</v>
       </c>
-      <c r="F26" s="15" t="n">
+      <c r="F26" s="16" t="n">
         <f aca="false">B26*(C26+$B$6)*$B$5</f>
         <v>1512</v>
       </c>
-      <c r="G26" s="15" t="n">
+      <c r="G26" s="16" t="n">
         <f aca="false">E26*(1+$B$7)</f>
         <v>1540</v>
       </c>
-      <c r="H26" s="16"/>
+      <c r="H26" s="17" t="n">
+        <v>27</v>
+      </c>
       <c r="I26" s="15" t="n">
         <f aca="false">B26*IF(H26="",C26,H26)*$B$5</f>
-        <v>1400</v>
+        <v>1512</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K26" s="15" t="n">
+        <f aca="false">B26*IF(J26="",IF(H26="",C26,H26),J26)*$B$5</f>
+        <v>1512</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="18" t="n">
+      <c r="A27" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D27" s="20" t="n">
+      <c r="D27" s="19" t="n">
         <f aca="false">B27*C27</f>
         <v>50</v>
       </c>
-      <c r="E27" s="21" t="n">
+      <c r="E27" s="20" t="n">
         <f aca="false">D27*$B$5</f>
         <v>1400</v>
       </c>
-      <c r="F27" s="22" t="n">
+      <c r="F27" s="21" t="n">
         <f aca="false">B27*(C27+$B$6)*$B$5</f>
         <v>1512</v>
       </c>
-      <c r="G27" s="22" t="n">
+      <c r="G27" s="21" t="n">
         <f aca="false">E27*(1+$B$7)</f>
         <v>1540</v>
       </c>
-      <c r="H27" s="16"/>
-      <c r="I27" s="22" t="n">
+      <c r="H27" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="I27" s="20" t="n">
         <f aca="false">B27*IF(H27="",C27,H27)*$B$5</f>
-        <v>1400</v>
+        <v>1512</v>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K27" s="20" t="n">
+        <f aca="false">B27*IF(J27="",IF(H27="",C27,H27),J27)*$B$5</f>
+        <v>1512</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="11" t="n">
+      <c r="A28" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C28" s="12" t="n">
+      <c r="C28" s="13" t="n">
         <v>21</v>
       </c>
-      <c r="D28" s="13" t="n">
+      <c r="D28" s="14" t="n">
         <f aca="false">B28*C28</f>
         <v>42</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="15" t="n">
         <f aca="false">D28*$B$5</f>
         <v>1176</v>
       </c>
-      <c r="F28" s="15" t="n">
+      <c r="F28" s="16" t="n">
         <f aca="false">B28*(C28+$B$6)*$B$5</f>
         <v>1288</v>
       </c>
-      <c r="G28" s="15" t="n">
+      <c r="G28" s="16" t="n">
         <f aca="false">E28*(1+$B$7)</f>
         <v>1293.6</v>
       </c>
-      <c r="H28" s="16"/>
+      <c r="H28" s="17" t="n">
+        <v>23</v>
+      </c>
       <c r="I28" s="15" t="n">
         <f aca="false">B28*IF(H28="",C28,H28)*$B$5</f>
-        <v>1176</v>
+        <v>1288</v>
+      </c>
+      <c r="J28" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="K28" s="15" t="n">
+        <f aca="false">B28*IF(J28="",IF(H28="",C28,H28),J28)*$B$5</f>
+        <v>1400</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" s="18" t="n">
+      <c r="A29" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D29" s="20" t="n">
+      <c r="D29" s="19" t="n">
         <f aca="false">B29*C29</f>
         <v>25</v>
       </c>
-      <c r="E29" s="21" t="n">
+      <c r="E29" s="20" t="n">
         <f aca="false">D29*$B$5</f>
         <v>700</v>
       </c>
-      <c r="F29" s="22" t="n">
+      <c r="F29" s="21" t="n">
         <f aca="false">B29*(C29+$B$6)*$B$5</f>
         <v>756</v>
       </c>
-      <c r="G29" s="22" t="n">
+      <c r="G29" s="21" t="n">
         <f aca="false">E29*(1+$B$7)</f>
         <v>770</v>
       </c>
-      <c r="H29" s="16"/>
-      <c r="I29" s="22" t="n">
+      <c r="H29" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="I29" s="20" t="n">
         <f aca="false">B29*IF(H29="",C29,H29)*$B$5</f>
-        <v>700</v>
+        <v>756</v>
+      </c>
+      <c r="J29" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K29" s="20" t="n">
+        <f aca="false">B29*IF(J29="",IF(H29="",C29,H29),J29)*$B$5</f>
+        <v>756</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" s="11" t="n">
+      <c r="A30" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C30" s="13" t="n">
         <v>21</v>
       </c>
-      <c r="D30" s="13" t="n">
+      <c r="D30" s="14" t="n">
         <f aca="false">B30*C30</f>
         <v>21</v>
       </c>
-      <c r="E30" s="14" t="n">
+      <c r="E30" s="15" t="n">
         <f aca="false">D30*$B$5</f>
         <v>588</v>
       </c>
-      <c r="F30" s="15" t="n">
+      <c r="F30" s="16" t="n">
         <f aca="false">B30*(C30+$B$6)*$B$5</f>
         <v>644</v>
       </c>
-      <c r="G30" s="15" t="n">
+      <c r="G30" s="16" t="n">
         <f aca="false">E30*(1+$B$7)</f>
         <v>646.8</v>
       </c>
-      <c r="H30" s="16"/>
+      <c r="H30" s="17" t="n">
+        <v>23</v>
+      </c>
       <c r="I30" s="15" t="n">
         <f aca="false">B30*IF(H30="",C30,H30)*$B$5</f>
-        <v>588</v>
+        <v>644</v>
+      </c>
+      <c r="J30" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="K30" s="15" t="n">
+        <f aca="false">B30*IF(J30="",IF(H30="",C30,H30),J30)*$B$5</f>
+        <v>644</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="18" t="n">
+      <c r="A31" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C31" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="D31" s="20" t="n">
+      <c r="D31" s="19" t="n">
         <f aca="false">B31*C31</f>
         <v>30</v>
       </c>
-      <c r="E31" s="21" t="n">
+      <c r="E31" s="20" t="n">
         <f aca="false">D31*$B$5</f>
         <v>840</v>
       </c>
-      <c r="F31" s="22" t="n">
+      <c r="F31" s="21" t="n">
         <f aca="false">B31*(C31+$B$6)*$B$5</f>
         <v>896</v>
       </c>
-      <c r="G31" s="22" t="n">
+      <c r="G31" s="21" t="n">
         <f aca="false">E31*(1+$B$7)</f>
         <v>924</v>
       </c>
-      <c r="H31" s="16"/>
-      <c r="I31" s="22" t="n">
+      <c r="H31" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="I31" s="20" t="n">
         <f aca="false">B31*IF(H31="",C31,H31)*$B$5</f>
         <v>840</v>
       </c>
+      <c r="J31" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K31" s="20" t="n">
+        <f aca="false">B31*IF(J31="",IF(H31="",C31,H31),J31)*$B$5</f>
+        <v>840</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="24" t="n">
+      <c r="A32" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="23" t="n">
         <f aca="false">SUM(B10:B31)</f>
         <v>180</v>
       </c>
-      <c r="C32" s="25"/>
-      <c r="D32" s="26" t="n">
+      <c r="C32" s="24"/>
+      <c r="D32" s="25" t="n">
         <f aca="false">SUM(D10:D31)</f>
         <v>5228.5</v>
       </c>
-      <c r="E32" s="25" t="n">
+      <c r="E32" s="24" t="n">
         <f aca="false">SUM(E10:E31)</f>
         <v>146398</v>
       </c>
-      <c r="F32" s="25" t="n">
+      <c r="F32" s="24" t="n">
         <f aca="false">SUM(F10:F31)</f>
         <v>156478</v>
       </c>
-      <c r="G32" s="25" t="n">
+      <c r="G32" s="24" t="n">
         <f aca="false">SUM(G10:G31)</f>
         <v>161037.8</v>
       </c>
-      <c r="H32" s="25"/>
-      <c r="I32" s="25" t="n">
+      <c r="H32" s="24"/>
+      <c r="I32" s="24" t="n">
         <f aca="false">SUM(I10:I31)</f>
-        <v>146398</v>
+        <v>150304</v>
+      </c>
+      <c r="J32" s="24"/>
+      <c r="K32" s="24" t="n">
+        <f aca="false">SUM(K10:K31)</f>
+        <v>159264</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28" t="n">
+      <c r="A33" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27" t="n">
         <f aca="false">F32-$E$32</f>
         <v>10080</v>
       </c>
-      <c r="G33" s="28" t="n">
+      <c r="G33" s="27" t="n">
         <f aca="false">G32-$E$32</f>
         <v>14639.8</v>
       </c>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28" t="n">
+      <c r="H33" s="27"/>
+      <c r="I33" s="27" t="n">
         <f aca="false">I32-$E$32</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29" t="s">
-        <v>39</v>
+        <v>3906</v>
+      </c>
+      <c r="J33" s="27"/>
+      <c r="K33" s="27" t="n">
+        <f aca="false">K32-$E$32</f>
+        <v>12866</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" s="27"/>
+      <c r="C34" s="27"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
+      <c r="I34" s="27"/>
+      <c r="J34" s="27"/>
+      <c r="K34" s="27" t="n">
+        <f aca="false">K32-$I$32</f>
+        <v>8960</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="30" t="s">
-        <v>40</v>
+      <c r="A36" s="28" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="30" t="s">
-        <v>41</v>
+      <c r="A37" s="29" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="30" t="s">
-        <v>42</v>
+      <c r="A38" s="29" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="30" t="s">
-        <v>43</v>
+      <c r="A39" s="29" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="30" t="s">
-        <v>44</v>
+      <c r="A40" s="29" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="30" t="s">
-        <v>45</v>
+      <c r="A41" s="29" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="29" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="29" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A9:I31"/>
+  <autoFilter ref="A9:K31"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>

</xml_diff>